<commit_message>
Commit after 15 placed
</commit_message>
<xml_diff>
--- a/DepartmentalStatus.xlsx
+++ b/DepartmentalStatus.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28224"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://indianinstituteofscience-my.sharepoint.com/personal/subhasisbisw_iisc_ac_in/Documents/PlacementExperiences/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="11_F25DC773A252ABDACC10487AE1DC6BBC5ADE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47DD7515-CB8E-402F-A911-0B63BC245AB8}"/>
+  <xr:revisionPtr revIDLastSave="111" documentId="11_F25DC773A252ABDACC10487AE1DC6BBC5ADE58EC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{82175AE1-690F-4DE3-8384-A104C582D6FA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="66">
   <si>
     <t>Sr No</t>
   </si>
@@ -182,6 +182,81 @@
   </si>
   <si>
     <t>Observe Ai MLE NLP</t>
+  </si>
+  <si>
+    <t>Vivek Dhamale</t>
+  </si>
+  <si>
+    <t>Fujitsu</t>
+  </si>
+  <si>
+    <t>AI Lab Researcher</t>
+  </si>
+  <si>
+    <t>25/28</t>
+  </si>
+  <si>
+    <t>Sameeksha Bhatia</t>
+  </si>
+  <si>
+    <t>Kevin Kuriakose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fujitsu </t>
+  </si>
+  <si>
+    <t>Monaka HPC</t>
+  </si>
+  <si>
+    <t>Ruchi Bhoot</t>
+  </si>
+  <si>
+    <t>FTI</t>
+  </si>
+  <si>
+    <t>Boddapati V S Dhruthi</t>
+  </si>
+  <si>
+    <t>Lam Research</t>
+  </si>
+  <si>
+    <t>ML Engineer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sudhanshu Pandey </t>
+  </si>
+  <si>
+    <t>Netradyne</t>
+  </si>
+  <si>
+    <t>Diksha Seth</t>
+  </si>
+  <si>
+    <t>18/24</t>
+  </si>
+  <si>
+    <t>Netradyne(DataScientist)</t>
+  </si>
+  <si>
+    <t>Arun Joshua Kennedy</t>
+  </si>
+  <si>
+    <t>AI engineer</t>
+  </si>
+  <si>
+    <t>Sofia Sunam</t>
+  </si>
+  <si>
+    <t>Sequential</t>
+  </si>
+  <si>
+    <t>Airtel</t>
+  </si>
+  <si>
+    <t>26/26</t>
+  </si>
+  <si>
+    <t>Data_Scientist_Airtel</t>
   </si>
 </sst>
 </file>
@@ -533,11 +608,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I7"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:I16"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.7109375" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="22.28515625" style="2" customWidth="1"/>
     <col min="3" max="3" width="25.28515625" style="2" customWidth="1"/>
     <col min="4" max="4" width="22.28515625" style="2" customWidth="1"/>
     <col min="5" max="6" width="22.7109375" style="2" customWidth="1"/>
@@ -749,6 +824,216 @@
         <v>40</v>
       </c>
     </row>
+    <row r="8" spans="1:9">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="3">
+        <v>45589</v>
+      </c>
+      <c r="D8" s="2">
+        <v>2</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="3">
+        <v>45589</v>
+      </c>
+      <c r="D9" s="2">
+        <v>2</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="3">
+        <v>45589</v>
+      </c>
+      <c r="D10" s="2">
+        <v>2</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="3">
+        <v>45589</v>
+      </c>
+      <c r="D11" s="2">
+        <v>2</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="3">
+        <v>45589</v>
+      </c>
+      <c r="D12" s="2">
+        <v>2</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" s="3">
+        <v>45591</v>
+      </c>
+      <c r="D13" s="2">
+        <v>2</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" s="3">
+        <v>45591</v>
+      </c>
+      <c r="D14" s="2">
+        <v>2</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="3">
+        <v>45591</v>
+      </c>
+      <c r="D15" s="2">
+        <v>2</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="3">
+        <v>45603</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="I4" r:id="rId1" display="../../../../:b:/g/personal/subhasisbisw_iisc_ac_in/EdJ6J2i--AlFp_HVz7NagcYBgB_1NXpN2o5Jh2563e611g?e=AbraDg" xr:uid="{9112A735-41E2-4A3F-BEF1-A918248E2F9B}"/>
@@ -756,8 +1041,9 @@
     <hyperlink ref="I3" r:id="rId3" display="../../../../:b:/g/personal/subhasisbisw_iisc_ac_in/EYchSqdumqFCpn2dryxqrroBqFtrXPCZkAL86EUzChG5lA?e=DLgcMr" xr:uid="{482EDA00-1E12-46F0-8CF2-96692A5E122E}"/>
     <hyperlink ref="I7" r:id="rId4" xr:uid="{3FB6B28F-DEAD-472B-BB2A-2446C965BB11}"/>
     <hyperlink ref="I6" r:id="rId5" xr:uid="{516740FD-F6A5-4DE9-85C1-57F0EE94AD35}"/>
+    <hyperlink ref="I14" r:id="rId6" xr:uid="{98064C19-299B-48A8-8E7B-DEF5F77B89EA}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId6"/>
+  <pageSetup orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>